<commit_message>
initial testing of createPregnancyCohort()
</commit_message>
<xml_diff>
--- a/tests/testthat/testCases/Test_data.xlsx
+++ b/tests/testthat/testCases/Test_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ginberg/Code/P4-C5-004/extras/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aalamshahi/Packages/PETConnector/tests/testthat/testCases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5451B2BB-27CB-8E49-90A6-98912CCAC774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB4FEBBA-364C-684F-809C-C7781F311CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="800" yWindow="2120" windowWidth="33760" windowHeight="20180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10700" yWindow="1200" windowWidth="21900" windowHeight="15040" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="95">
   <si>
     <t>person_id</t>
   </si>
@@ -324,6 +324,9 @@
   </si>
   <si>
     <t>pregnancy_outcome</t>
+  </si>
+  <si>
+    <t>Mother to test duplicate map</t>
   </si>
 </sst>
 </file>
@@ -744,7 +747,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="4" width="35.5" customWidth="1"/>
@@ -1273,7 +1276,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>100</v>
       </c>
@@ -1299,8 +1302,45 @@
         <v>40</v>
       </c>
     </row>
+    <row r="22" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
+        <v>102</v>
+      </c>
+      <c r="B22" s="1">
+        <v>8532</v>
+      </c>
+      <c r="C22" s="1">
+        <v>1</v>
+      </c>
+      <c r="D22" s="1">
+        <v>6</v>
+      </c>
+      <c r="E22" s="1">
+        <v>2000</v>
+      </c>
+      <c r="F22" s="1">
+        <v>0</v>
+      </c>
+      <c r="G22" s="1">
+        <v>0</v>
+      </c>
+      <c r="H22" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="F23" s="1"/>
+    </row>
     <row r="24" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="E24" s="1"/>
       <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="4"/>
+      <c r="L24" s="4"/>
     </row>
     <row r="25" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
@@ -1332,8 +1372,6 @@
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
-      <c r="I27" s="4"/>
-      <c r="L27" s="4"/>
     </row>
     <row r="28" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
@@ -1344,15 +1382,6 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
     </row>
-    <row r="29" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1360,7 +1389,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB104438-4099-6E40-90B1-739F61573A13}">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="18.6640625" customWidth="1"/>
@@ -1923,6 +1952,64 @@
       </c>
       <c r="K17" s="1"/>
     </row>
+    <row r="18" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
+        <v>102</v>
+      </c>
+      <c r="B18" s="1">
+        <v>71</v>
+      </c>
+      <c r="C18" s="10">
+        <v>44296</v>
+      </c>
+      <c r="D18" s="10">
+        <v>44568</v>
+      </c>
+      <c r="E18" s="1">
+        <v>270</v>
+      </c>
+      <c r="F18" s="1">
+        <v>4092289</v>
+      </c>
+      <c r="G18" s="1">
+        <v>4015701</v>
+      </c>
+      <c r="H18" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="I18" s="1">
+        <v>4188539</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
+        <v>102</v>
+      </c>
+      <c r="B19" s="1">
+        <v>72</v>
+      </c>
+      <c r="C19" s="10">
+        <v>44296</v>
+      </c>
+      <c r="D19" s="10">
+        <v>44568</v>
+      </c>
+      <c r="E19" s="1">
+        <v>270</v>
+      </c>
+      <c r="F19" s="1">
+        <v>4092289</v>
+      </c>
+      <c r="G19" s="1">
+        <v>4015701</v>
+      </c>
+      <c r="H19" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="I19" s="1">
+        <v>4188539</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J17">
     <sortCondition ref="G1:G17"/>
@@ -1933,7 +2020,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2B8B433-8712-6348-9439-118BA945D9FC}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.1640625" bestFit="1" customWidth="1"/>
@@ -2363,6 +2450,23 @@
         <v>40</v>
       </c>
     </row>
+    <row r="22" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
+        <v>102</v>
+      </c>
+      <c r="B22" s="1">
+        <v>102</v>
+      </c>
+      <c r="C22" s="6">
+        <v>38718</v>
+      </c>
+      <c r="D22" s="6">
+        <v>45657</v>
+      </c>
+      <c r="E22" s="1">
+        <v>32880</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2370,7 +2474,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EED5A0E5-6553-46ED-AC90-012DDE271310}">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="18.1640625" bestFit="1" customWidth="1"/>
@@ -2792,6 +2896,46 @@
       </c>
       <c r="G18" s="4" t="s">
         <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A19" s="4">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4">
+        <v>102</v>
+      </c>
+      <c r="C19" s="11">
+        <v>4145947</v>
+      </c>
+      <c r="D19" s="12">
+        <v>44743</v>
+      </c>
+      <c r="E19" s="12">
+        <v>44743</v>
+      </c>
+      <c r="F19" s="11">
+        <v>32820</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A20" s="4">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4">
+        <v>103</v>
+      </c>
+      <c r="C20" s="11">
+        <v>4145947</v>
+      </c>
+      <c r="D20" s="12">
+        <v>44744</v>
+      </c>
+      <c r="E20" s="12">
+        <v>44806</v>
+      </c>
+      <c r="F20" s="11">
+        <v>32821</v>
       </c>
     </row>
   </sheetData>
@@ -3853,7 +3997,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5BBCCA6-1E90-4542-A320-9B59DFDDE9AE}">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" customWidth="1"/>
@@ -4137,21 +4281,64 @@
         <v>62</v>
       </c>
     </row>
+    <row r="11" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>72</v>
+      </c>
+      <c r="B11" s="1">
+        <v>17</v>
+      </c>
+      <c r="C11" s="1">
+        <v>17</v>
+      </c>
+      <c r="D11">
+        <v>4092289</v>
+      </c>
+      <c r="E11" s="1">
+        <v>4000</v>
+      </c>
+      <c r="F11" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="G11" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="H11" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>71</v>
+      </c>
+      <c r="B12" s="1">
+        <v>18</v>
+      </c>
+      <c r="C12" s="1">
+        <v>18</v>
+      </c>
+      <c r="D12">
+        <v>4092289</v>
+      </c>
+      <c r="E12" s="1">
+        <v>4000</v>
+      </c>
+      <c r="F12" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="G12" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="H12" s="1">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f696df8-7461-455e-9bf1-ef56149775f2">
@@ -4161,7 +4348,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005E48E57FAF33F44FB5E762D78C70B43B" ma:contentTypeVersion="9" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="09261b8c9db6496040fa98c128102db7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2f696df8-7461-455e-9bf1-ef56149775f2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c87049393a058ff896145aa7aaeb09f0" ns2:_="">
     <xsd:import namespace="2f696df8-7461-455e-9bf1-ef56149775f2"/>
@@ -4333,15 +4520,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F405B8-D94E-404D-BACC-4EAF448A1B08}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DDF05F8-3308-4EA3-8F5D-FC78E20AC719}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -4357,7 +4545,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C331738-2870-4EAF-86B4-6F4811A40645}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4373,4 +4561,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F405B8-D94E-404D-BACC-4EAF448A1B08}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update filtering of duplicate children from fact_relationship
1. In the case of identical rows, reduce records to one record per subject

2. After the above scenario has been resolved, if there is still >1 of the same subject_id, all records with that subject_id will be filtered out
</commit_message>
<xml_diff>
--- a/tests/testthat/testCases/Test_data.xlsx
+++ b/tests/testthat/testCases/Test_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aalamshahi/Packages/PETConnector/tests/testthat/testCases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB4FEBBA-364C-684F-809C-C7781F311CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F9FE03-AECB-BD43-9C37-25B97F4AE4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10700" yWindow="1200" windowWidth="21900" windowHeight="15040" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,9 @@
     <sheet name="measurement" sheetId="7" r:id="rId6"/>
     <sheet name="infant" sheetId="4" r:id="rId7"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">fact_relationship!$A$1:$F$46</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="98">
   <si>
     <t>person_id</t>
   </si>
@@ -327,6 +330,15 @@
   </si>
   <si>
     <t>Mother to test duplicate map</t>
+  </si>
+  <si>
+    <t>Family 5- Stillbirth, duplicate</t>
+  </si>
+  <si>
+    <t>Twin to infant 18. Duplicate to preg 72/inf 17</t>
+  </si>
+  <si>
+    <t>Family 4- Infant of Mother, duplicate</t>
   </si>
 </sst>
 </file>
@@ -2945,7 +2957,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7613E543-FC05-4844-9753-12567E4D8F20}">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" style="2" customWidth="1"/>
@@ -2977,23 +2989,23 @@
       <c r="G1" s="4"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="5">
-        <v>1147314</v>
-      </c>
-      <c r="B2" s="4">
+      <c r="A2" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D2">
         <v>1</v>
-      </c>
-      <c r="C2" s="5">
-        <v>1147314</v>
-      </c>
-      <c r="D2" s="4">
-        <v>3</v>
       </c>
       <c r="E2">
         <v>40485452</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -3001,19 +3013,19 @@
         <v>1147314</v>
       </c>
       <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D3">
         <v>1</v>
-      </c>
-      <c r="C3" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="D3">
-        <v>4</v>
       </c>
       <c r="E3">
         <v>40485452</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -3021,19 +3033,19 @@
         <v>1147314</v>
       </c>
       <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D4">
         <v>1</v>
       </c>
-      <c r="C4" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="D4">
-        <v>5</v>
-      </c>
       <c r="E4">
-        <v>4285883</v>
+        <v>40485452</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -3041,19 +3053,19 @@
         <v>1147314</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" s="3">
         <v>1147314</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -3061,19 +3073,19 @@
         <v>1147314</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C6" s="3">
         <v>1147314</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E6">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -3081,19 +3093,19 @@
         <v>1147314</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C7" s="3">
         <v>1147314</v>
       </c>
       <c r="D7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E7">
-        <v>4285883</v>
+        <v>4326600</v>
       </c>
       <c r="F7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -3107,13 +3119,13 @@
         <v>1147314</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8">
         <v>40485452</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -3121,7 +3133,7 @@
         <v>1147314</v>
       </c>
       <c r="B9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" s="3">
         <v>1147314</v>
@@ -3141,19 +3153,19 @@
         <v>1147314</v>
       </c>
       <c r="B10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C10" s="3">
         <v>1147314</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10">
         <v>40485452</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -3161,7 +3173,7 @@
         <v>1147314</v>
       </c>
       <c r="B11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C11" s="3">
         <v>1147314</v>
@@ -3170,7 +3182,7 @@
         <v>2</v>
       </c>
       <c r="E11">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F11" t="s">
         <v>31</v>
@@ -3181,19 +3193,19 @@
         <v>1147314</v>
       </c>
       <c r="B12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C12" s="3">
         <v>1147314</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -3210,30 +3222,30 @@
         <v>2</v>
       </c>
       <c r="E13">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F13" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="B14">
-        <v>6</v>
-      </c>
-      <c r="C14" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="D14">
-        <v>7</v>
+      <c r="A14" s="5">
+        <v>1147314</v>
+      </c>
+      <c r="B14" s="4">
+        <v>1</v>
+      </c>
+      <c r="C14" s="5">
+        <v>1147314</v>
+      </c>
+      <c r="D14" s="4">
+        <v>3</v>
       </c>
       <c r="E14">
-        <v>4285883</v>
+        <v>40485452</v>
       </c>
       <c r="F14" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -3241,39 +3253,39 @@
         <v>1147314</v>
       </c>
       <c r="B15">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C15" s="3">
         <v>1147314</v>
       </c>
       <c r="D15">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E15">
         <v>40485452</v>
       </c>
       <c r="F15" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="B16">
-        <v>7</v>
-      </c>
-      <c r="C16" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="D16">
-        <v>6</v>
+      <c r="A16" s="5">
+        <v>1147314</v>
+      </c>
+      <c r="B16" s="4">
+        <v>1</v>
+      </c>
+      <c r="C16" s="5">
+        <v>1147314</v>
+      </c>
+      <c r="D16" s="4">
+        <v>3</v>
       </c>
       <c r="E16">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F16" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -3281,19 +3293,19 @@
         <v>1147314</v>
       </c>
       <c r="B17">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C17" s="3">
         <v>1147314</v>
       </c>
       <c r="D17">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E17">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F17" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -3301,19 +3313,19 @@
         <v>1147314</v>
       </c>
       <c r="B18">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C18" s="3">
         <v>1147314</v>
       </c>
       <c r="D18">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E18">
         <v>40485452</v>
       </c>
       <c r="F18" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -3321,19 +3333,19 @@
         <v>1147314</v>
       </c>
       <c r="B19">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C19" s="3">
         <v>1147314</v>
       </c>
       <c r="D19">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E19">
         <v>40485452</v>
       </c>
       <c r="F19" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -3341,19 +3353,19 @@
         <v>1147314</v>
       </c>
       <c r="B20">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C20" s="3">
         <v>1147314</v>
       </c>
       <c r="D20">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E20">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F20" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -3361,19 +3373,19 @@
         <v>1147314</v>
       </c>
       <c r="B21">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C21" s="3">
         <v>1147314</v>
       </c>
       <c r="D21">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E21">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F21" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -3381,19 +3393,19 @@
         <v>1147314</v>
       </c>
       <c r="B22">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="C22" s="3">
         <v>1147314</v>
       </c>
       <c r="D22">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E22">
-        <v>40485452</v>
+        <v>4285883</v>
       </c>
       <c r="F22" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -3401,33 +3413,33 @@
         <v>1147314</v>
       </c>
       <c r="B23">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="C23" s="3">
         <v>1147314</v>
       </c>
       <c r="D23">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E23">
         <v>4285883</v>
       </c>
       <c r="F23" t="s">
-        <v>61</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="5">
-        <v>1147314</v>
-      </c>
-      <c r="B24" s="4">
+      <c r="A24" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="B24">
         <v>1</v>
       </c>
-      <c r="C24" s="5">
-        <v>1147314</v>
-      </c>
-      <c r="D24" s="4">
-        <v>3</v>
+      <c r="C24" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D24">
+        <v>5</v>
       </c>
       <c r="E24">
         <v>4326600</v>
@@ -3441,19 +3453,19 @@
         <v>1147314</v>
       </c>
       <c r="B25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" s="3">
         <v>1147314</v>
       </c>
       <c r="D25">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E25">
         <v>4326600</v>
       </c>
       <c r="F25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -3461,19 +3473,19 @@
         <v>1147314</v>
       </c>
       <c r="B26">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C26" s="3">
         <v>1147314</v>
       </c>
       <c r="D26">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E26">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F26" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -3481,19 +3493,19 @@
         <v>1147314</v>
       </c>
       <c r="B27">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C27" s="3">
         <v>1147314</v>
       </c>
       <c r="D27">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E27">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F27" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -3501,19 +3513,19 @@
         <v>1147314</v>
       </c>
       <c r="B28">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C28" s="3">
         <v>1147314</v>
       </c>
       <c r="D28">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E28">
         <v>4326600</v>
       </c>
       <c r="F28" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
@@ -3521,19 +3533,19 @@
         <v>1147314</v>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C29" s="3">
         <v>1147314</v>
       </c>
       <c r="D29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E29">
         <v>4326600</v>
       </c>
       <c r="F29" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -3541,19 +3553,19 @@
         <v>1147314</v>
       </c>
       <c r="B30">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C30" s="3">
         <v>1147314</v>
       </c>
       <c r="D30">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E30">
-        <v>4326600</v>
+        <v>4285883</v>
       </c>
       <c r="F30" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
@@ -3561,19 +3573,19 @@
         <v>1147314</v>
       </c>
       <c r="B31">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C31" s="3">
         <v>1147314</v>
       </c>
       <c r="D31">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E31">
         <v>4326600</v>
       </c>
       <c r="F31" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
@@ -3581,19 +3593,19 @@
         <v>1147314</v>
       </c>
       <c r="B32">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C32" s="3">
         <v>1147314</v>
       </c>
       <c r="D32">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E32">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F32" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -3601,19 +3613,19 @@
         <v>1147314</v>
       </c>
       <c r="B33">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C33" s="3">
         <v>1147314</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E33">
         <v>4326600</v>
       </c>
       <c r="F33" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
@@ -3621,19 +3633,19 @@
         <v>1147314</v>
       </c>
       <c r="B34">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C34" s="3">
         <v>1147314</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E34">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F34" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
@@ -3641,19 +3653,19 @@
         <v>1147314</v>
       </c>
       <c r="B35">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C35" s="3">
         <v>1147314</v>
       </c>
       <c r="D35">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E35">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F35" t="s">
-        <v>31</v>
+        <v>97</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -3661,19 +3673,19 @@
         <v>1147314</v>
       </c>
       <c r="B36">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C36" s="3">
         <v>1147314</v>
       </c>
       <c r="D36">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E36">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F36" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -3681,19 +3693,19 @@
         <v>1147314</v>
       </c>
       <c r="B37">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C37" s="3">
         <v>1147314</v>
       </c>
       <c r="D37">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E37">
         <v>4326600</v>
       </c>
       <c r="F37" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
@@ -3701,19 +3713,19 @@
         <v>1147314</v>
       </c>
       <c r="B38">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C38" s="3">
         <v>1147314</v>
       </c>
       <c r="D38">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E38">
         <v>4326600</v>
       </c>
       <c r="F38" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -3721,19 +3733,19 @@
         <v>1147314</v>
       </c>
       <c r="B39">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C39" s="3">
         <v>1147314</v>
       </c>
       <c r="D39">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E39">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F39" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -3770,7 +3782,7 @@
         <v>13</v>
       </c>
       <c r="E41">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F41" t="s">
         <v>43</v>
@@ -3781,19 +3793,19 @@
         <v>1147314</v>
       </c>
       <c r="B42">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C42" s="3">
         <v>1147314</v>
       </c>
       <c r="D42">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E42">
         <v>4326600</v>
       </c>
       <c r="F42" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
@@ -3801,19 +3813,19 @@
         <v>1147314</v>
       </c>
       <c r="B43">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C43" s="3">
         <v>1147314</v>
       </c>
       <c r="D43">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E43">
-        <v>4326600</v>
+        <v>4285883</v>
       </c>
       <c r="F43" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -3821,19 +3833,19 @@
         <v>1147314</v>
       </c>
       <c r="B44">
+        <v>15</v>
+      </c>
+      <c r="C44" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D44">
         <v>14</v>
-      </c>
-      <c r="C44" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="D44">
-        <v>15</v>
       </c>
       <c r="E44">
         <v>4326600</v>
       </c>
       <c r="F44" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
@@ -3841,19 +3853,39 @@
         <v>1147314</v>
       </c>
       <c r="B45">
+        <v>14</v>
+      </c>
+      <c r="C45" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D45">
         <v>15</v>
       </c>
-      <c r="C45" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="D45">
+      <c r="E45">
+        <v>40485452</v>
+      </c>
+      <c r="F45" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="B46">
         <v>14</v>
       </c>
-      <c r="E45">
+      <c r="C46" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D46">
+        <v>15</v>
+      </c>
+      <c r="E46">
         <v>4326600</v>
       </c>
-      <c r="F45" t="s">
-        <v>61</v>
+      <c r="F46" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -3997,7 +4029,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5BBCCA6-1E90-4542-A320-9B59DFDDE9AE}">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" customWidth="1"/>
@@ -4248,74 +4280,69 @@
       <c r="D9">
         <v>443213</v>
       </c>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
       <c r="I9" s="4" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="1">
-        <v>16</v>
+        <v>111</v>
       </c>
       <c r="C10" s="1">
-        <v>16</v>
+        <v>111</v>
       </c>
       <c r="D10">
         <v>443213</v>
       </c>
-      <c r="E10" s="1">
-        <v>3000</v>
-      </c>
-      <c r="F10" s="1">
-        <v>4188539</v>
-      </c>
-      <c r="G10" s="1">
-        <v>4188539</v>
-      </c>
-      <c r="H10" s="1">
-        <v>7</v>
-      </c>
       <c r="I10" s="4" t="s">
-        <v>62</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
-        <v>72</v>
+        <v>9</v>
       </c>
       <c r="B11" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D11">
-        <v>4092289</v>
+        <v>443213</v>
       </c>
       <c r="E11" s="1">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="F11" s="1">
-        <v>4188540</v>
+        <v>4188539</v>
       </c>
       <c r="G11" s="1">
-        <v>4188540</v>
+        <v>4188539</v>
       </c>
       <c r="H11" s="1">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B12" s="1">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" s="1">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D12">
         <v>4092289</v>
@@ -4330,6 +4357,62 @@
         <v>4188540</v>
       </c>
       <c r="H12" s="1">
+        <v>10</v>
+      </c>
+      <c r="I12" s="4"/>
+    </row>
+    <row r="13" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>71</v>
+      </c>
+      <c r="B13" s="1">
+        <v>17</v>
+      </c>
+      <c r="C13" s="1">
+        <v>17</v>
+      </c>
+      <c r="D13">
+        <v>4092289</v>
+      </c>
+      <c r="E13" s="1">
+        <v>4000</v>
+      </c>
+      <c r="F13" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="G13" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="H13" s="1">
+        <v>10</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
+        <v>71</v>
+      </c>
+      <c r="B14" s="1">
+        <v>18</v>
+      </c>
+      <c r="C14" s="1">
+        <v>18</v>
+      </c>
+      <c r="D14">
+        <v>4092289</v>
+      </c>
+      <c r="E14" s="1">
+        <v>4000</v>
+      </c>
+      <c r="F14" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="G14" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="H14" s="1">
         <v>10</v>
       </c>
     </row>
@@ -4339,16 +4422,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f696df8-7461-455e-9bf1-ef56149775f2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005E48E57FAF33F44FB5E762D78C70B43B" ma:contentTypeVersion="9" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="09261b8c9db6496040fa98c128102db7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2f696df8-7461-455e-9bf1-ef56149775f2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c87049393a058ff896145aa7aaeb09f0" ns2:_="">
     <xsd:import namespace="2f696df8-7461-455e-9bf1-ef56149775f2"/>
@@ -4520,6 +4593,16 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f696df8-7461-455e-9bf1-ef56149775f2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -4530,22 +4613,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DDF05F8-3308-4EA3-8F5D-FC78E20AC719}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="2f696df8-7461-455e-9bf1-ef56149775f2"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C331738-2870-4EAF-86B4-6F4811A40645}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4563,6 +4630,22 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DDF05F8-3308-4EA3-8F5D-FC78E20AC719}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="2f696df8-7461-455e-9bf1-ef56149775f2"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F405B8-D94E-404D-BACC-4EAF448A1B08}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Added a test for filterLiveBirth() when creating from fact_relationship table
1. Added a family 6 to fact_relationship, person, and observation period table for child 25/mom 30 in the xlsx

2. To the pregnancy_cohort created in setup.R, added a pregnancy for mom 30/pregnancy 27 to not affect the createPregnancyCohort.R tests
</commit_message>
<xml_diff>
--- a/tests/testthat/testCases/Test_data.xlsx
+++ b/tests/testthat/testCases/Test_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aalamshahi/Packages/PETConnector/tests/testthat/testCases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF9A2423-CEF7-1D45-A634-D7E00B86B6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E5FB4E-0F35-2744-BE87-C2B5EFEE932B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20240" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5340" yWindow="760" windowWidth="34560" windowHeight="20220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="infant" sheetId="4" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">fact_relationship!$A$1:$F$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">fact_relationship!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="101">
   <si>
     <t>person_id</t>
   </si>
@@ -342,6 +342,12 @@
   </si>
   <si>
     <t>Family 4 - Twin 2, "bad" duplicate</t>
+  </si>
+  <si>
+    <t>Family 6- Infant of Mother</t>
+  </si>
+  <si>
+    <t>Family 6 - daughter</t>
   </si>
 </sst>
 </file>
@@ -1344,7 +1350,30 @@
       </c>
     </row>
     <row r="23" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="F23" s="1"/>
+      <c r="A23" s="1">
+        <v>25</v>
+      </c>
+      <c r="B23" s="1">
+        <v>8532</v>
+      </c>
+      <c r="C23" s="1">
+        <v>1</v>
+      </c>
+      <c r="D23" s="1">
+        <v>7</v>
+      </c>
+      <c r="E23" s="1">
+        <v>2022</v>
+      </c>
+      <c r="F23" s="1">
+        <v>0</v>
+      </c>
+      <c r="G23" s="1">
+        <v>0</v>
+      </c>
+      <c r="H23" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="24" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
@@ -2035,7 +2064,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2B8B433-8712-6348-9439-118BA945D9FC}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.1640625" bestFit="1" customWidth="1"/>
@@ -2500,6 +2529,26 @@
       </c>
       <c r="E23" s="1">
         <v>32880</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>25</v>
+      </c>
+      <c r="B24" s="1">
+        <v>25</v>
+      </c>
+      <c r="C24" s="7">
+        <v>44568</v>
+      </c>
+      <c r="D24" s="8">
+        <v>45657</v>
+      </c>
+      <c r="E24" s="1">
+        <v>32880</v>
+      </c>
+      <c r="F24" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2980,7 +3029,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7613E543-FC05-4844-9753-12567E4D8F20}">
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" style="2" customWidth="1"/>
@@ -3016,19 +3065,19 @@
         <v>1147314</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2" s="3">
         <v>1147314</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>40485452</v>
+        <v>4285883</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -3036,19 +3085,19 @@
         <v>1147314</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3" s="3">
         <v>1147314</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E3">
-        <v>40485452</v>
+        <v>4285883</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -3056,19 +3105,19 @@
         <v>1147314</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3">
         <v>1147314</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E4">
-        <v>40485452</v>
+        <v>4285883</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -3076,19 +3125,19 @@
         <v>1147314</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="3">
         <v>1147314</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E5">
-        <v>4326600</v>
+        <v>4285883</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -3096,7 +3145,7 @@
         <v>1147314</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" s="3">
         <v>1147314</v>
@@ -3116,7 +3165,7 @@
         <v>1147314</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7" s="3">
         <v>1147314</v>
@@ -3136,19 +3185,19 @@
         <v>1147314</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C8" s="3">
         <v>1147314</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -3156,7 +3205,7 @@
         <v>1147314</v>
       </c>
       <c r="B9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" s="3">
         <v>1147314</v>
@@ -3165,7 +3214,7 @@
         <v>2</v>
       </c>
       <c r="E9">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F9" t="s">
         <v>31</v>
@@ -3176,7 +3225,7 @@
         <v>1147314</v>
       </c>
       <c r="B10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" s="3">
         <v>1147314</v>
@@ -3185,7 +3234,7 @@
         <v>2</v>
       </c>
       <c r="E10">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F10" t="s">
         <v>31</v>
@@ -3196,7 +3245,7 @@
         <v>1147314</v>
       </c>
       <c r="B11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C11" s="3">
         <v>1147314</v>
@@ -3212,23 +3261,23 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="B12">
-        <v>4</v>
-      </c>
-      <c r="C12" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="D12">
-        <v>2</v>
+      <c r="A12" s="5">
+        <v>1147314</v>
+      </c>
+      <c r="B12" s="4">
+        <v>1</v>
+      </c>
+      <c r="C12" s="5">
+        <v>1147314</v>
+      </c>
+      <c r="D12" s="4">
+        <v>3</v>
       </c>
       <c r="E12">
         <v>4326600</v>
       </c>
       <c r="F12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -3236,36 +3285,36 @@
         <v>1147314</v>
       </c>
       <c r="B13">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C13" s="3">
         <v>1147314</v>
       </c>
       <c r="D13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13">
         <v>4326600</v>
       </c>
       <c r="F13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="5">
-        <v>1147314</v>
-      </c>
-      <c r="B14" s="4">
+      <c r="A14" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="B14">
         <v>1</v>
       </c>
-      <c r="C14" s="5">
-        <v>1147314</v>
-      </c>
-      <c r="D14" s="4">
-        <v>3</v>
+      <c r="C14" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D14">
+        <v>4</v>
       </c>
       <c r="E14">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F14" t="s">
         <v>28</v>
@@ -3282,27 +3331,27 @@
         <v>1147314</v>
       </c>
       <c r="D15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F15" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="5">
-        <v>1147314</v>
-      </c>
-      <c r="B16" s="4">
+      <c r="A16" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="B16">
         <v>1</v>
       </c>
-      <c r="C16" s="5">
-        <v>1147314</v>
-      </c>
-      <c r="D16" s="4">
-        <v>3</v>
+      <c r="C16" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
       </c>
       <c r="E16">
         <v>4326600</v>
@@ -3322,7 +3371,7 @@
         <v>1147314</v>
       </c>
       <c r="D17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E17">
         <v>4326600</v>
@@ -3336,19 +3385,19 @@
         <v>1147314</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C18" s="3">
         <v>1147314</v>
       </c>
       <c r="D18">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E18">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F18" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -3356,19 +3405,19 @@
         <v>1147314</v>
       </c>
       <c r="B19">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C19" s="3">
         <v>1147314</v>
       </c>
       <c r="D19">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E19">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F19" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -3376,19 +3425,19 @@
         <v>1147314</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C20" s="3">
         <v>1147314</v>
       </c>
       <c r="D20">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E20">
         <v>4326600</v>
       </c>
       <c r="F20" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -3396,19 +3445,19 @@
         <v>1147314</v>
       </c>
       <c r="B21">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C21" s="3">
         <v>1147314</v>
       </c>
       <c r="D21">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E21">
         <v>4326600</v>
       </c>
       <c r="F21" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -3416,19 +3465,19 @@
         <v>1147314</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C22" s="3">
         <v>1147314</v>
       </c>
       <c r="D22">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E22">
-        <v>4285883</v>
+        <v>4326600</v>
       </c>
       <c r="F22" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -3436,19 +3485,19 @@
         <v>1147314</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C23" s="3">
         <v>1147314</v>
       </c>
       <c r="D23">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E23">
-        <v>4285883</v>
+        <v>4326600</v>
       </c>
       <c r="F23" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
@@ -3456,19 +3505,19 @@
         <v>1147314</v>
       </c>
       <c r="B24">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C24" s="3">
         <v>1147314</v>
       </c>
       <c r="D24">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E24">
         <v>4326600</v>
       </c>
       <c r="F24" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -3476,19 +3525,19 @@
         <v>1147314</v>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C25" s="3">
         <v>1147314</v>
       </c>
       <c r="D25">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E25">
         <v>4326600</v>
       </c>
       <c r="F25" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -3496,19 +3545,19 @@
         <v>1147314</v>
       </c>
       <c r="B26">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C26" s="3">
         <v>1147314</v>
       </c>
       <c r="D26">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E26">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F26" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -3516,19 +3565,19 @@
         <v>1147314</v>
       </c>
       <c r="B27">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C27" s="3">
         <v>1147314</v>
       </c>
       <c r="D27">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E27">
-        <v>40485452</v>
+        <v>4326600</v>
       </c>
       <c r="F27" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -3536,19 +3585,19 @@
         <v>1147314</v>
       </c>
       <c r="B28">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C28" s="3">
         <v>1147314</v>
       </c>
       <c r="D28">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E28">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F28" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
@@ -3556,19 +3605,19 @@
         <v>1147314</v>
       </c>
       <c r="B29">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C29" s="3">
         <v>1147314</v>
       </c>
       <c r="D29">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E29">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F29" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -3576,19 +3625,19 @@
         <v>1147314</v>
       </c>
       <c r="B30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C30" s="3">
         <v>1147314</v>
       </c>
       <c r="D30">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E30">
-        <v>4285883</v>
+        <v>40485452</v>
       </c>
       <c r="F30" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
@@ -3596,19 +3645,19 @@
         <v>1147314</v>
       </c>
       <c r="B31">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C31" s="3">
         <v>1147314</v>
       </c>
       <c r="D31">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E31">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F31" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
@@ -3616,19 +3665,19 @@
         <v>1147314</v>
       </c>
       <c r="B32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C32" s="3">
         <v>1147314</v>
       </c>
       <c r="D32">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E32">
         <v>40485452</v>
       </c>
       <c r="F32" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -3636,39 +3685,39 @@
         <v>1147314</v>
       </c>
       <c r="B33">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C33" s="3">
         <v>1147314</v>
       </c>
       <c r="D33">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E33">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F33" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A34" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="B34">
-        <v>12</v>
-      </c>
-      <c r="C34" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="D34">
-        <v>11</v>
+      <c r="A34" s="5">
+        <v>1147314</v>
+      </c>
+      <c r="B34" s="4">
+        <v>1</v>
+      </c>
+      <c r="C34" s="5">
+        <v>1147314</v>
+      </c>
+      <c r="D34" s="4">
+        <v>3</v>
       </c>
       <c r="E34">
         <v>40485452</v>
       </c>
       <c r="F34" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
@@ -3676,19 +3725,19 @@
         <v>1147314</v>
       </c>
       <c r="B35">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C35" s="3">
         <v>1147314</v>
       </c>
       <c r="D35">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E35">
         <v>40485452</v>
       </c>
       <c r="F35" t="s">
-        <v>97</v>
+        <v>29</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -3696,19 +3745,19 @@
         <v>1147314</v>
       </c>
       <c r="B36">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C36" s="3">
         <v>1147314</v>
       </c>
       <c r="D36">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E36">
         <v>40485452</v>
       </c>
       <c r="F36" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -3716,19 +3765,19 @@
         <v>1147314</v>
       </c>
       <c r="B37">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C37" s="3">
         <v>1147314</v>
       </c>
       <c r="D37">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E37">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F37" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
@@ -3736,19 +3785,19 @@
         <v>1147314</v>
       </c>
       <c r="B38">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C38" s="3">
         <v>1147314</v>
       </c>
       <c r="D38">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E38">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F38" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -3756,19 +3805,19 @@
         <v>1147314</v>
       </c>
       <c r="B39">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C39" s="3">
         <v>1147314</v>
       </c>
       <c r="D39">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E39">
         <v>40485452</v>
       </c>
       <c r="F39" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -3776,19 +3825,19 @@
         <v>1147314</v>
       </c>
       <c r="B40">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C40" s="3">
         <v>1147314</v>
       </c>
       <c r="D40">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E40">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F40" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
@@ -3796,19 +3845,19 @@
         <v>1147314</v>
       </c>
       <c r="B41">
+        <v>12</v>
+      </c>
+      <c r="C41" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D41">
         <v>11</v>
-      </c>
-      <c r="C41" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="D41">
-        <v>13</v>
       </c>
       <c r="E41">
         <v>40485452</v>
       </c>
       <c r="F41" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
@@ -3816,19 +3865,19 @@
         <v>1147314</v>
       </c>
       <c r="B42">
+        <v>12</v>
+      </c>
+      <c r="C42" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D42">
         <v>11</v>
       </c>
-      <c r="C42" s="3">
-        <v>1147314</v>
-      </c>
-      <c r="D42">
-        <v>13</v>
-      </c>
       <c r="E42">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F42" t="s">
-        <v>43</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
@@ -3836,19 +3885,19 @@
         <v>1147314</v>
       </c>
       <c r="B43">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C43" s="3">
         <v>1147314</v>
       </c>
       <c r="D43">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E43">
-        <v>4285883</v>
+        <v>40485452</v>
       </c>
       <c r="F43" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -3856,19 +3905,19 @@
         <v>1147314</v>
       </c>
       <c r="B44">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C44" s="3">
         <v>1147314</v>
       </c>
       <c r="D44">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E44">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F44" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
@@ -3876,19 +3925,19 @@
         <v>1147314</v>
       </c>
       <c r="B45">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C45" s="3">
         <v>1147314</v>
       </c>
       <c r="D45">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E45">
         <v>40485452</v>
       </c>
       <c r="F45" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
@@ -3905,13 +3954,34 @@
         <v>15</v>
       </c>
       <c r="E46">
-        <v>4326600</v>
+        <v>40485452</v>
       </c>
       <c r="F46" t="s">
         <v>60</v>
       </c>
     </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="B47">
+        <v>25</v>
+      </c>
+      <c r="C47" s="3">
+        <v>1147314</v>
+      </c>
+      <c r="D47">
+        <v>30</v>
+      </c>
+      <c r="E47">
+        <v>40485452</v>
+      </c>
+      <c r="F47" t="s">
+        <v>99</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{7613E543-FC05-4844-9753-12567E4D8F20}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4455,6 +4525,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005E48E57FAF33F44FB5E762D78C70B43B" ma:contentTypeVersion="9" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="09261b8c9db6496040fa98c128102db7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2f696df8-7461-455e-9bf1-ef56149775f2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c87049393a058ff896145aa7aaeb09f0" ns2:_="">
     <xsd:import namespace="2f696df8-7461-455e-9bf1-ef56149775f2"/>
@@ -4626,15 +4705,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DDF05F8-3308-4EA3-8F5D-FC78E20AC719}">
   <ds:schemaRefs>
@@ -4652,6 +4722,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F405B8-D94E-404D-BACC-4EAF448A1B08}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C331738-2870-4EAF-86B4-6F4811A40645}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4667,12 +4745,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F405B8-D94E-404D-BACC-4EAF448A1B08}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
added test case for distinct but overlapping pregnancies for same birthing parent
</commit_message>
<xml_diff>
--- a/tests/testthat/testCases/Test_data.xlsx
+++ b/tests/testthat/testCases/Test_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aalamshahi/Packages/PETConnector/tests/testthat/testCases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E5FB4E-0F35-2744-BE87-C2B5EFEE932B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57FE672E-255F-9249-8235-19325C7B2540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5340" yWindow="760" windowWidth="34560" windowHeight="20220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36520" yWindow="700" windowWidth="30780" windowHeight="19680" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="102">
   <si>
     <t>person_id</t>
   </si>
@@ -348,6 +348,9 @@
   </si>
   <si>
     <t>Family 6 - daughter</t>
+  </si>
+  <si>
+    <t>Mother to test overlap of distinct pregnancies</t>
   </si>
 </sst>
 </file>
@@ -768,7 +771,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="4" width="35.5" customWidth="1"/>
@@ -1376,13 +1379,30 @@
       </c>
     </row>
     <row r="24" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
+      <c r="A24" s="1">
+        <v>104</v>
+      </c>
+      <c r="B24" s="1">
+        <v>8532</v>
+      </c>
+      <c r="C24" s="1">
+        <v>1</v>
+      </c>
+      <c r="D24" s="1">
+        <v>6</v>
+      </c>
+      <c r="E24" s="1">
+        <v>1992</v>
+      </c>
+      <c r="F24" s="1">
+        <v>0</v>
+      </c>
+      <c r="G24" s="1">
+        <v>0</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>101</v>
+      </c>
       <c r="I24" s="4"/>
       <c r="L24" s="4"/>
     </row>
@@ -1405,8 +1425,6 @@
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
-      <c r="I26" s="4"/>
-      <c r="L26" s="4"/>
     </row>
     <row r="27" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
@@ -1417,15 +1435,6 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
     </row>
-    <row r="28" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1433,7 +1442,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB104438-4099-6E40-90B1-739F61573A13}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="18.6640625" customWidth="1"/>
@@ -2054,6 +2063,70 @@
         <v>4188539</v>
       </c>
     </row>
+    <row r="20" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
+        <v>104</v>
+      </c>
+      <c r="B20" s="1">
+        <v>43</v>
+      </c>
+      <c r="C20" s="10">
+        <v>43832</v>
+      </c>
+      <c r="D20" s="10">
+        <v>44089</v>
+      </c>
+      <c r="E20" s="1">
+        <v>270</v>
+      </c>
+      <c r="F20" s="1">
+        <v>4092289</v>
+      </c>
+      <c r="G20" s="1">
+        <v>4015701</v>
+      </c>
+      <c r="H20" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="I20" s="1">
+        <v>4188539</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
+        <v>104</v>
+      </c>
+      <c r="B21" s="1">
+        <v>44</v>
+      </c>
+      <c r="C21" s="10">
+        <v>43840</v>
+      </c>
+      <c r="D21" s="10">
+        <v>44094</v>
+      </c>
+      <c r="E21" s="1">
+        <v>270</v>
+      </c>
+      <c r="F21" s="1">
+        <v>4092289</v>
+      </c>
+      <c r="G21" s="1">
+        <v>4015701</v>
+      </c>
+      <c r="H21" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="I21" s="1">
+        <v>4188539</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J17">
     <sortCondition ref="G1:G17"/>
@@ -2064,7 +2137,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2B8B433-8712-6348-9439-118BA945D9FC}">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.1640625" bestFit="1" customWidth="1"/>
@@ -2549,6 +2622,26 @@
       </c>
       <c r="F24" t="s">
         <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
+        <v>104</v>
+      </c>
+      <c r="B25" s="1">
+        <v>104</v>
+      </c>
+      <c r="C25" s="6">
+        <v>38718</v>
+      </c>
+      <c r="D25" s="6">
+        <v>45657</v>
+      </c>
+      <c r="E25" s="1">
+        <v>32880</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dropping pregnancies with identical IDs but differing dates, overlapping or not
</commit_message>
<xml_diff>
--- a/tests/testthat/testCases/Test_data.xlsx
+++ b/tests/testthat/testCases/Test_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aalamshahi/Packages/PETConnector/tests/testthat/testCases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57FE672E-255F-9249-8235-19325C7B2540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7744FFA-DDD3-A544-AAA3-3D90AFBA8B96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36520" yWindow="700" windowWidth="30780" windowHeight="19680" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36520" yWindow="700" windowWidth="30780" windowHeight="19680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="104">
   <si>
     <t>person_id</t>
   </si>
@@ -351,6 +351,12 @@
   </si>
   <si>
     <t>Mother to test overlap of distinct pregnancies</t>
+  </si>
+  <si>
+    <t>Mother to test identical pregnancy ID and overlapping dates</t>
+  </si>
+  <si>
+    <t>Mother to test identical pregnancy ID and non-overlapping dates</t>
   </si>
 </sst>
 </file>
@@ -771,7 +777,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="4" width="35.5" customWidth="1"/>
@@ -1407,24 +1413,60 @@
       <c r="L24" s="4"/>
     </row>
     <row r="25" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
+      <c r="A25" s="1">
+        <v>105</v>
+      </c>
+      <c r="B25" s="1">
+        <v>8532</v>
+      </c>
+      <c r="C25" s="1">
+        <v>1</v>
+      </c>
+      <c r="D25" s="1">
+        <v>6</v>
+      </c>
+      <c r="E25" s="1">
+        <v>1992</v>
+      </c>
+      <c r="F25" s="1">
+        <v>0</v>
+      </c>
+      <c r="G25" s="1">
+        <v>0</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>102</v>
+      </c>
       <c r="I25" s="4"/>
       <c r="L25" s="4"/>
     </row>
     <row r="26" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
+      <c r="A26" s="1">
+        <v>106</v>
+      </c>
+      <c r="B26" s="1">
+        <v>8532</v>
+      </c>
+      <c r="C26" s="1">
+        <v>1</v>
+      </c>
+      <c r="D26" s="1">
+        <v>6</v>
+      </c>
+      <c r="E26" s="1">
+        <v>1992</v>
+      </c>
+      <c r="F26" s="1">
+        <v>0</v>
+      </c>
+      <c r="G26" s="1">
+        <v>0</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="I26" s="4"/>
+      <c r="L26" s="4"/>
     </row>
     <row r="27" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
@@ -1435,6 +1477,15 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
     </row>
+    <row r="28" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1442,7 +1493,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB104438-4099-6E40-90B1-739F61573A13}">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="18.6640625" customWidth="1"/>
@@ -2127,6 +2178,166 @@
         <v>101</v>
       </c>
     </row>
+    <row r="22" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
+        <v>105</v>
+      </c>
+      <c r="B22" s="1">
+        <v>45</v>
+      </c>
+      <c r="C22" s="10">
+        <v>43840</v>
+      </c>
+      <c r="D22" s="10">
+        <v>44094</v>
+      </c>
+      <c r="E22" s="1">
+        <v>270</v>
+      </c>
+      <c r="F22" s="1">
+        <v>4092289</v>
+      </c>
+      <c r="G22" s="1">
+        <v>4015701</v>
+      </c>
+      <c r="H22" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="I22" s="1">
+        <v>4188539</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
+        <v>105</v>
+      </c>
+      <c r="B23" s="1">
+        <v>45</v>
+      </c>
+      <c r="C23" s="10">
+        <v>43832</v>
+      </c>
+      <c r="D23" s="10">
+        <v>44089</v>
+      </c>
+      <c r="E23" s="1">
+        <v>270</v>
+      </c>
+      <c r="F23" s="1">
+        <v>4092289</v>
+      </c>
+      <c r="G23" s="1">
+        <v>4015701</v>
+      </c>
+      <c r="H23" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="I23" s="1">
+        <v>4188539</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>105</v>
+      </c>
+      <c r="B24" s="1">
+        <v>45</v>
+      </c>
+      <c r="C24" s="10">
+        <v>43845</v>
+      </c>
+      <c r="D24" s="10">
+        <v>44101</v>
+      </c>
+      <c r="E24" s="1">
+        <v>270</v>
+      </c>
+      <c r="F24" s="1">
+        <v>4092289</v>
+      </c>
+      <c r="G24" s="1">
+        <v>4015701</v>
+      </c>
+      <c r="H24" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="I24" s="1">
+        <v>4188539</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
+        <v>106</v>
+      </c>
+      <c r="B25" s="1">
+        <v>46</v>
+      </c>
+      <c r="C25" s="10">
+        <v>43832</v>
+      </c>
+      <c r="D25" s="10">
+        <v>44089</v>
+      </c>
+      <c r="E25" s="1">
+        <v>270</v>
+      </c>
+      <c r="F25" s="1">
+        <v>4092289</v>
+      </c>
+      <c r="G25" s="1">
+        <v>4015701</v>
+      </c>
+      <c r="H25" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="I25" s="1">
+        <v>4188539</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
+        <v>106</v>
+      </c>
+      <c r="B26" s="1">
+        <v>46</v>
+      </c>
+      <c r="C26" s="10">
+        <v>42005</v>
+      </c>
+      <c r="D26" s="10">
+        <v>42248</v>
+      </c>
+      <c r="E26" s="1">
+        <v>270</v>
+      </c>
+      <c r="F26" s="1">
+        <v>4092289</v>
+      </c>
+      <c r="G26" s="1">
+        <v>4015701</v>
+      </c>
+      <c r="H26" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="I26" s="1">
+        <v>4188539</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J17">
     <sortCondition ref="G1:G17"/>
@@ -2137,7 +2348,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2B8B433-8712-6348-9439-118BA945D9FC}">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.1640625" bestFit="1" customWidth="1"/>
@@ -2642,6 +2853,46 @@
       </c>
       <c r="F25" s="1" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
+        <v>105</v>
+      </c>
+      <c r="B26" s="1">
+        <v>105</v>
+      </c>
+      <c r="C26" s="6">
+        <v>38718</v>
+      </c>
+      <c r="D26" s="6">
+        <v>45657</v>
+      </c>
+      <c r="E26" s="1">
+        <v>32880</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
+        <v>106</v>
+      </c>
+      <c r="B27" s="1">
+        <v>106</v>
+      </c>
+      <c r="C27" s="6">
+        <v>38718</v>
+      </c>
+      <c r="D27" s="6">
+        <v>45657</v>
+      </c>
+      <c r="E27" s="1">
+        <v>32880</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -4608,25 +4859,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f696df8-7461-455e-9bf1-ef56149775f2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005E48E57FAF33F44FB5E762D78C70B43B" ma:contentTypeVersion="9" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="09261b8c9db6496040fa98c128102db7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2f696df8-7461-455e-9bf1-ef56149775f2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c87049393a058ff896145aa7aaeb09f0" ns2:_="">
     <xsd:import namespace="2f696df8-7461-455e-9bf1-ef56149775f2"/>
@@ -4798,31 +5030,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DDF05F8-3308-4EA3-8F5D-FC78E20AC719}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="2f696df8-7461-455e-9bf1-ef56149775f2"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F405B8-D94E-404D-BACC-4EAF448A1B08}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f696df8-7461-455e-9bf1-ef56149775f2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C331738-2870-4EAF-86B4-6F4811A40645}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4838,4 +5065,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F405B8-D94E-404D-BACC-4EAF448A1B08}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DDF05F8-3308-4EA3-8F5D-FC78E20AC719}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="2f696df8-7461-455e-9bf1-ef56149775f2"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
introduction of samePregDiffDates argument for createPregnancyCohort()
</commit_message>
<xml_diff>
--- a/tests/testthat/testCases/Test_data.xlsx
+++ b/tests/testthat/testCases/Test_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aalamshahi/Packages/PETConnector/tests/testthat/testCases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7744FFA-DDD3-A544-AAA3-3D90AFBA8B96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AAFC3E6-64C3-FB4F-863B-E0D542FACB17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36520" yWindow="700" windowWidth="30780" windowHeight="19680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="160" yWindow="940" windowWidth="17040" windowHeight="19920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="104">
   <si>
     <t>person_id</t>
   </si>
@@ -1493,7 +1493,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB104438-4099-6E40-90B1-739F61573A13}">
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="18.6640625" customWidth="1"/>
@@ -2250,10 +2250,10 @@
         <v>45</v>
       </c>
       <c r="C24" s="10">
-        <v>43845</v>
+        <v>43832</v>
       </c>
       <c r="D24" s="10">
-        <v>44101</v>
+        <v>44090</v>
       </c>
       <c r="E24" s="1">
         <v>270</v>
@@ -2276,16 +2276,16 @@
     </row>
     <row r="25" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B25" s="1">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C25" s="10">
-        <v>43832</v>
+        <v>43845</v>
       </c>
       <c r="D25" s="10">
-        <v>44089</v>
+        <v>44101</v>
       </c>
       <c r="E25" s="1">
         <v>270</v>
@@ -2303,7 +2303,7 @@
         <v>4188539</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -2314,10 +2314,10 @@
         <v>46</v>
       </c>
       <c r="C26" s="10">
-        <v>42005</v>
+        <v>43832</v>
       </c>
       <c r="D26" s="10">
-        <v>42248</v>
+        <v>44089</v>
       </c>
       <c r="E26" s="1">
         <v>270</v>
@@ -2335,6 +2335,38 @@
         <v>4188539</v>
       </c>
       <c r="J26" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
+        <v>106</v>
+      </c>
+      <c r="B27" s="1">
+        <v>46</v>
+      </c>
+      <c r="C27" s="10">
+        <v>42005</v>
+      </c>
+      <c r="D27" s="10">
+        <v>42248</v>
+      </c>
+      <c r="E27" s="1">
+        <v>270</v>
+      </c>
+      <c r="F27" s="1">
+        <v>4092289</v>
+      </c>
+      <c r="G27" s="1">
+        <v>4015701</v>
+      </c>
+      <c r="H27" s="1">
+        <v>4188540</v>
+      </c>
+      <c r="I27" s="1">
+        <v>4188539</v>
+      </c>
+      <c r="J27" s="1" t="s">
         <v>103</v>
       </c>
     </row>
@@ -5031,15 +5063,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f696df8-7461-455e-9bf1-ef56149775f2">
@@ -5047,6 +5070,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5068,14 +5100,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F405B8-D94E-404D-BACC-4EAF448A1B08}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DDF05F8-3308-4EA3-8F5D-FC78E20AC719}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -5089,4 +5113,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F405B8-D94E-404D-BACC-4EAF448A1B08}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>